<commit_message>
Align template quantity labels and add format download dropdown
</commit_message>
<xml_diff>
--- a/pricing-upload-template.xlsx
+++ b/pricing-upload-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selling Prices" sheetId="1" r:id="R36a49f5fbfcf4360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selling Prices" sheetId="1" r:id="R2f019d7ba7da4584"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,11 +51,14 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -262,49 +265,57 @@
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="19" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="48" customHeight="1">
+      <x:c r="A1" s="4" t="str">
         <x:v>SKU</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="4" t="str">
         <x:v>Card Product Name</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="4" t="str">
         <x:v>Price Type</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>QTY 0</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>QTY 5,000</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>QTY 10,000</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>QTY 25,000</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>QTY 50,000</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
-        <x:v>QTY 100,000</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="str">
-        <x:v>QTY 250,000</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="str">
-        <x:v>QTY 500,000</x:v>
+      <x:c r="D1" s="4" t="str">
+        <x:v>QTY 0
+1–4,999</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>QTY 5,000
+5,000–9,999</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>QTY 10,000
+10,000–24,999</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>QTY 25,000
+25,000–49,999</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>QTY 50,000
+50,000–99,999</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>QTY 100,000
+100,000–249,999</x:v>
+      </x:c>
+      <x:c r="J1" s="4" t="str">
+        <x:v>QTY 250,000
+250,000–499,999</x:v>
+      </x:c>
+      <x:c r="K1" s="4" t="str">
+        <x:v>QTY 500,000
+500,000+</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
@@ -313,14 +324,14 @@
       <x:c r="C2" s="1" t="str">
         <x:v>Standard Price (EMEA License)</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="str"/>
-      <x:c r="E2" s="4" t="str"/>
-      <x:c r="F2" s="4" t="str"/>
-      <x:c r="G2" s="4" t="str"/>
-      <x:c r="H2" s="4" t="str"/>
-      <x:c r="I2" s="4" t="str"/>
-      <x:c r="J2" s="4" t="str"/>
-      <x:c r="K2" s="4" t="str"/>
+      <x:c r="D2" s="5" t="str"/>
+      <x:c r="E2" s="5" t="str"/>
+      <x:c r="F2" s="5" t="str"/>
+      <x:c r="G2" s="5" t="str"/>
+      <x:c r="H2" s="5" t="str"/>
+      <x:c r="I2" s="5" t="str"/>
+      <x:c r="J2" s="5" t="str"/>
+      <x:c r="K2" s="5" t="str"/>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="1" t="str"/>
@@ -328,14 +339,14 @@
       <x:c r="C3" s="1" t="str">
         <x:v>Base Price (EMEA Premium)</x:v>
       </x:c>
-      <x:c r="D3" s="4" t="str"/>
-      <x:c r="E3" s="4" t="str"/>
-      <x:c r="F3" s="4" t="str"/>
-      <x:c r="G3" s="4" t="str"/>
-      <x:c r="H3" s="4" t="str"/>
-      <x:c r="I3" s="4" t="str"/>
-      <x:c r="J3" s="4" t="str"/>
-      <x:c r="K3" s="4" t="str"/>
+      <x:c r="D3" s="5" t="str"/>
+      <x:c r="E3" s="5" t="str"/>
+      <x:c r="F3" s="5" t="str"/>
+      <x:c r="G3" s="5" t="str"/>
+      <x:c r="H3" s="5" t="str"/>
+      <x:c r="I3" s="5" t="str"/>
+      <x:c r="J3" s="5" t="str"/>
+      <x:c r="K3" s="5" t="str"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="1" t="str"/>
@@ -343,14 +354,14 @@
       <x:c r="C4" s="1" t="str">
         <x:v>Distributor Price (EMEA)</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="str"/>
-      <x:c r="E4" s="4" t="str"/>
-      <x:c r="F4" s="4" t="str"/>
-      <x:c r="G4" s="4" t="str"/>
-      <x:c r="H4" s="4" t="str"/>
-      <x:c r="I4" s="4" t="str"/>
-      <x:c r="J4" s="4" t="str"/>
-      <x:c r="K4" s="4" t="str"/>
+      <x:c r="D4" s="5" t="str"/>
+      <x:c r="E4" s="5" t="str"/>
+      <x:c r="F4" s="5" t="str"/>
+      <x:c r="G4" s="5" t="str"/>
+      <x:c r="H4" s="5" t="str"/>
+      <x:c r="I4" s="5" t="str"/>
+      <x:c r="J4" s="5" t="str"/>
+      <x:c r="K4" s="5" t="str"/>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
       <x:c r="A5" s="1" t="str"/>
@@ -358,14 +369,14 @@
       <x:c r="C5" s="1" t="str">
         <x:v>EMEA Strategic Account (MAF)</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="str"/>
-      <x:c r="E5" s="4" t="str"/>
-      <x:c r="F5" s="4" t="str"/>
-      <x:c r="G5" s="4" t="str"/>
-      <x:c r="H5" s="4" t="str"/>
-      <x:c r="I5" s="4" t="str"/>
-      <x:c r="J5" s="4" t="str"/>
-      <x:c r="K5" s="4" t="str"/>
+      <x:c r="D5" s="5" t="str"/>
+      <x:c r="E5" s="5" t="str"/>
+      <x:c r="F5" s="5" t="str"/>
+      <x:c r="G5" s="5" t="str"/>
+      <x:c r="H5" s="5" t="str"/>
+      <x:c r="I5" s="5" t="str"/>
+      <x:c r="J5" s="5" t="str"/>
+      <x:c r="K5" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>